<commit_message>
fix(validator): multi-domain default gate + H4 confidence + regression pins (W0)
- validate_data.py CLI now validates EVERY registered domain by default
  (slug-prefixed, aggregated); --data-dir narrows. Closes the structural
  gap that let PAM/IGA defects pass a 'clean' secrets-only run.
- check_ownership_sources now enforces the documented confidence contract
  (HIGH/MEDIUM/LOW required on dated acquisition edges) — H4 completion.
- Regression pins for the closed REG-F1 / IGA-F1 / PAM-SME-01 defects.
- CI simplified to the single multi-domain call.
- Stakeholder XLSX sheet titles/readme compute counts from live data
  (was hardcoded 47/37; data is 50/37); pack regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stakeholder/Secrets-Mgmt-Stakeholder-Pack-2026-06-03.xlsx
+++ b/stakeholder/Secrets-Mgmt-Stakeholder-Pack-2026-06-03.xlsx
@@ -8,13 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Use Cases (47)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Use Cases (50)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="NHI Taxonomy (37)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Regulatory back-map" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sources index" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Use Cases (47)'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Use Cases (50)'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NHI Taxonomy (37)'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Regulatory back-map'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources index'!$A$1:$C$1</definedName>
@@ -581,7 +581,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>matrix/use-cases.csv, matrix/identity-catalog.csv, matrix/regulatory-trace.csv (CSV data contracts; validate_data.py green; 111 tests pass).</t>
+          <t>matrix/domains/secrets/use-cases.csv, matrix/domains/secrets/identity-catalog.csv, matrix/domains/secrets/regulatory-trace.csv (CSV data contracts; gated by validate_data.py and the full pytest suite, both green at generation time).</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>47 use cases and 37 NHI types for enterprise secrets management, each linked to primary regulatory and standards sources. Audience: security, risk, audit and engineering stakeholders.</t>
+          <t>50 use cases and 37 NHI types for enterprise secrets management, each linked to primary regulatory and standards sources. Audience: security, risk, audit and engineering stakeholders.</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>CPS234-§15; CPS234-§21(a); CPS234-§21(d); CPS234-§23; CPS234-§24; CPS234-§26; CPS234-§35; ISM-0043; ISM-1401; ISM-1404; ISM-1437; ISM-1611; ISM-1613</t>
+          <t>CPS234-§15; CPS234-§21(a); CPS234-§21(d); CPS234-§23; CPS234-§24; CPS234-§26; CPS234-§35; ISM-0043; ISM-1401; ISM-1437; ISM-1611; ISM-1613</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024; csa-ai-agents-2024; astrix-nhi-report-2024</t>
+          <t>owasp-llm06-2025; csa-agentic-iam-2025; astrix-nhi-report-2024</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024</t>
+          <t>owasp-llm06-2025</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>CPS234-§17; CPS234-§21(c); ISM-0363; ISM-1613</t>
+          <t>CPS234-§17; CPS234-§21(c); ISM-0363; ISM-1404; ISM-1613</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>CPS234-§13; CPS234-§21(a); CPS234-§21(d); CPS234-§23; CPS234-§24; CPS234-§26; CPS234-§35; CPS234-§36; CPS230-§42; ISM-0043; ISM-0140; ISM-1404; ISM-1405; ISM-1611; ISM-1613</t>
+          <t>CPS234-§13; CPS234-§21(a); CPS234-§21(d); CPS234-§23; CPS234-§24; CPS234-§26; CPS234-§35; CPS234-§36; CPS230-§42; ISM-0043; ISM-0140; ISM-1405; ISM-1611; ISM-1613</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024; csa-ai-agents-2024; astrix-nhi-report-2024</t>
+          <t>owasp-llm06-2025; csa-agentic-iam-2025; astrix-nhi-report-2024</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024</t>
+          <t>owasp-llm06-2025</t>
         </is>
       </c>
     </row>
@@ -3530,6 +3530,177 @@
       <c r="K48" s="5" t="inlineStr">
         <is>
           <t>ibm-racf-2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>UC-F-028</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>FUNCTIONAL</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Agent credential issuance via broker</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>As a platform engineer I want autonomous AI agents to receive tool and API credentials only from a broker that mints per-session, per-tool, scoped, short-lived credentials, so that a compromised or prompt-injected agent cannot obtain or exfiltrate a long-lived secret.</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Static long-lived API keys for agents are forbidden in new patterns; agent credentials are broker-minted, scoped per tool and per session, and short-lived; every issuance is logged with the agent identity, owner and requesting purpose; issuance is denied to unregistered or unowned agents.</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>NHI-019; NHI-010</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>ZT-Pillar-Identity; ZT-Pillar-Workload; E8-RestrictAdminPriv</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>CPS234-§21; ISM-1619; LLM06:2025</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025; csa-agentic-iam-2025</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>UC-F-029</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>FUNCTIONAL</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Agent credential rotation &amp; revocation</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>As a secrets owner I want credentials held by autonomous agents to rotate automatically on a risk cadence and to be revoked immediately when an agent is decommissioned or shows signs of compromise, so that no agent credential outlives the agent's purpose or a containment event.</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Agent-held credentials rotate automatically on a risk-tiered cadence with no service interruption; decommissioning or compromise of an agent triggers immediate revocation of its issued credentials and active sessions; rotation/revocation coverage for agent identities is a tracked KPI and trends up; no long-lived static agent secret persists past its rotation window.</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>NHI-019; NHI-009; NHI-010</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>ZT-Pillar-Identity; ZT-Pillar-Workload</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>CPS234-§21; ISM-1619; LLM06:2025</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025; csa-agentic-iam-2025</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>UC-F-030</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>FUNCTIONAL</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Agent secret-scope confinement</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>As a risk owner I want every credential issued to an autonomous agent to be scoped to the minimum tools and data its declared task needs, and for over-broad agent secret-scope to be detected and flagged, so that excessive agency in the credential plane cannot translate a single agent compromise into broad lateral access.</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Agent credentials are scoped per task and per tool by default; over-broad or unused scopes on agent credentials are detected and flagged for right-sizing; scope grants are tied to the agent's declared purpose and owner; excessive-agency conditions (credential scope beyond declared purpose) are surfaced to the owner.</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>NHI-019</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>ZT-Pillar-Identity; E8-RestrictAdminPriv</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>CPS234-§21; LLM06:2025</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>owasp-llm06-2025</t>
         </is>
       </c>
     </row>
@@ -3583,6 +3754,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4640,12 +4814,12 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024; csa-ai-agents-2024; astrix-nhi-report-2024; nhimg-ultimate-guide-2025</t>
+          <t>owasp-llm06-2025; csa-agentic-iam-2025; astrix-nhi-report-2024; nhimg-ultimate-guide-2025</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024</t>
+          <t>owasp-llm06-2025</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6178,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>UC-F-001; UC-F-003; UC-F-004; UC-F-005; UC-F-006; UC-F-008; UC-F-009; UC-F-010; UC-F-012; UC-F-016; UC-F-018; UC-F-019; UC-F-020; UC-F-021; UC-F-022; UC-F-024</t>
+          <t>UC-F-001; UC-F-003; UC-F-004; UC-F-005; UC-F-006; UC-F-008; UC-F-009; UC-F-010; UC-F-012; UC-F-016; UC-F-018; UC-F-019; UC-F-020; UC-F-021; UC-F-022; UC-F-024; UC-F-028; UC-F-029; UC-F-030</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -7336,7 +7510,7 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>UC-F-001; UC-F-003; UC-F-004; UC-F-005; UC-F-006; UC-F-008; UC-F-009; UC-F-010; UC-F-012; UC-F-013; UC-F-015; UC-F-018; UC-F-020; UC-F-024; UC-F-025; UC-N-002; UC-N-019</t>
+          <t>UC-F-001; UC-F-003; UC-F-004; UC-F-005; UC-F-006; UC-F-008; UC-F-009; UC-F-010; UC-F-012; UC-F-013; UC-F-015; UC-F-018; UC-F-020; UC-F-024; UC-F-025; UC-N-002; UC-N-019; UC-F-028; UC-F-029</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
@@ -8076,7 +8250,7 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>UC-F-011; UC-F-018; UC-N-001; UC-N-011; UC-N-017; UC-N-019</t>
+          <t>UC-F-011; UC-F-018; UC-N-001; UC-N-011; UC-N-017; UC-N-019; UC-F-029</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
@@ -8182,12 +8356,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Suspension of access to systems (credential revocation)</t>
+          <t>Unprivileged inactive-account disablement at 45 days</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>UC-F-007; UC-N-011</t>
+          <t>UC-F-027</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -8604,7 +8778,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.cyber.gov.au/resources-business-and-government/essential-cybersecurity/essential-eight/essential-eight-maturity-model</t>
+          <t>https://www.cyber.gov.au/business-government/asds-cyber-security-frameworks/essential-eight/essential-eight-maturity-model</t>
         </is>
       </c>
     </row>
@@ -9155,17 +9329,17 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>csa-ai-agents-2024</t>
+          <t>csa-agentic-iam-2025</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Securing AI Agents and Agentic Workflows</t>
+          <t>Agentic AI Identity and Access Management: A New Approach</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>https://cloudsecurityalliance.org/research/topics/artificial-intelligence</t>
+          <t>https://cloudsecurityalliance.org/artifacts/agentic-ai-identity-and-access-management-a-new-approach</t>
         </is>
       </c>
     </row>
@@ -10192,17 +10366,17 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>owasp-llm-top10-2024</t>
+          <t>owasp-llm06-2025</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for Large Language Model Applications</t>
+          <t>OWASP Top 10 for LLM Applications — LLM06:2025 Excessive Agency</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>https://owasp.org/www-project-top-10-for-large-language-model-applications/</t>
+          <t>https://genai.owasp.org/llmrisk/llm062025-excessive-agency/</t>
         </is>
       </c>
     </row>

</xml_diff>